<commit_message>
adding rotor mass and surface area optimizer script, as output by Claude
</commit_message>
<xml_diff>
--- a/VehicleParameters.xlsx
+++ b/VehicleParameters.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\GitHub\RIT_RacingBrakesAnalysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC6FEEB4-F76C-4658-923E-5D3996E0B5A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B495F0F-15FE-490D-AC2A-5AE6B27A8A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="1" r:id="rId1"/>
     <sheet name="MuTable" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" fullCalcOnLoad="true"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="183" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="122">
   <si>
     <t>Name</t>
   </si>
@@ -405,8 +405,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -425,7 +425,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -433,15 +433,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -460,7 +458,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -611,7 +609,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="true">
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -635,9 +633,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="true">
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -661,7 +659,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -696,7 +694,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -714,7 +712,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="true">
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -739,7 +737,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -775,18 +773,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E47"/>
-  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.3046875" customWidth="true"/>
-    <col min="2" max="2" width="10" customWidth="true"/>
-    <col min="3" max="3" width="9.765625" customWidth="true"/>
-    <col min="4" max="4" width="17.61328125" customWidth="true"/>
-    <col min="5" max="5" width="120.69140625" customWidth="true"/>
+    <col min="1" max="1" width="21.3046875" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="9.765625" customWidth="1"/>
+    <col min="4" max="4" width="17.61328125" customWidth="1"/>
+    <col min="5" max="5" width="120.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -803,7 +801,7 @@
         <v>66</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -820,12 +818,12 @@
         <v>93</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>0.30753999999999998</v>
+        <v>0.11</v>
       </c>
       <c r="C3" t="s">
         <v>42</v>
@@ -837,7 +835,7 @@
         <v>92</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -854,7 +852,7 @@
         <v>67</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -871,7 +869,7 @@
         <v>68</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -888,7 +886,7 @@
         <v>69</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -905,7 +903,7 @@
         <v>70</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -922,7 +920,7 @@
         <v>71</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -939,7 +937,7 @@
         <v>72</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -956,7 +954,7 @@
         <v>94</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -973,7 +971,7 @@
         <v>73</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -987,7 +985,7 @@
         <v>59</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -1004,7 +1002,7 @@
         <v>74</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -1021,7 +1019,7 @@
         <v>75</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -1038,7 +1036,7 @@
         <v>76</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -1055,7 +1053,7 @@
         <v>95</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -1072,7 +1070,7 @@
         <v>96</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -1089,7 +1087,7 @@
         <v>77</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -1106,7 +1104,7 @@
         <v>78</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -1123,7 +1121,7 @@
         <v>79</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -1140,7 +1138,7 @@
         <v>80</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -1157,7 +1155,7 @@
         <v>81</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -1174,7 +1172,7 @@
         <v>82</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -1191,7 +1189,7 @@
         <v>97</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -1208,7 +1206,7 @@
         <v>98</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -1225,7 +1223,7 @@
         <v>83</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -1239,7 +1237,7 @@
         <v>56</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -1253,7 +1251,7 @@
         <v>56</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -1270,7 +1268,7 @@
         <v>84</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>29</v>
       </c>
@@ -1284,7 +1282,7 @@
         <v>56</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>30</v>
       </c>
@@ -1298,7 +1296,7 @@
         <v>56</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -1315,7 +1313,7 @@
         <v>85</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -1329,7 +1327,7 @@
         <v>65</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>33</v>
       </c>
@@ -1346,7 +1344,7 @@
         <v>86</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>34</v>
       </c>
@@ -1360,7 +1358,7 @@
         <v>65</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -1377,7 +1375,7 @@
         <v>87</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>36</v>
       </c>
@@ -1391,7 +1389,7 @@
         <v>65</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>37</v>
       </c>
@@ -1408,7 +1406,7 @@
         <v>88</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -1425,139 +1423,139 @@
         <v>89</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="0" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A40" t="s">
         <v>99</v>
       </c>
-      <c r="B40" s="0">
+      <c r="B40">
         <v>35</v>
       </c>
-      <c r="C40" s="0" t="s">
+      <c r="C40" t="s">
         <v>107</v>
       </c>
-      <c r="D40" s="0" t="s">
+      <c r="D40" t="s">
         <v>113</v>
       </c>
-      <c r="E40" s="0" t="s">
+      <c r="E40" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="0" t="s">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A41" t="s">
         <v>100</v>
       </c>
-      <c r="B41" s="0">
+      <c r="B41">
         <v>200</v>
       </c>
-      <c r="C41" s="0" t="s">
+      <c r="C41" t="s">
         <v>108</v>
       </c>
-      <c r="D41" s="0" t="s">
+      <c r="D41" t="s">
         <v>113</v>
       </c>
-      <c r="E41" s="0" t="s">
+      <c r="E41" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="0" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A42" t="s">
         <v>101</v>
       </c>
-      <c r="B42" s="0">
+      <c r="B42">
         <v>30000</v>
       </c>
-      <c r="C42" s="0" t="s">
+      <c r="C42" t="s">
         <v>109</v>
       </c>
-      <c r="D42" s="0" t="s">
+      <c r="D42" t="s">
         <v>113</v>
       </c>
-      <c r="E42" s="0" t="s">
+      <c r="E42" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="0" t="s">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A43" t="s">
         <v>102</v>
       </c>
-      <c r="B43" s="0">
+      <c r="B43">
         <v>7041</v>
       </c>
-      <c r="C43" s="0" t="s">
+      <c r="C43" t="s">
         <v>110</v>
       </c>
-      <c r="D43" s="0" t="s">
+      <c r="D43" t="s">
         <v>64</v>
       </c>
-      <c r="E43" s="0" t="s">
+      <c r="E43" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="0" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A44" t="s">
         <v>103</v>
       </c>
-      <c r="B44" s="0">
+      <c r="B44">
         <v>-0.93500000000000005</v>
       </c>
-      <c r="C44" s="0" t="s">
+      <c r="C44" t="s">
         <v>44</v>
       </c>
-      <c r="D44" s="0" t="s">
+      <c r="D44" t="s">
         <v>64</v>
       </c>
-      <c r="E44" s="0" t="s">
+      <c r="E44" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="0" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A45" t="s">
         <v>104</v>
       </c>
-      <c r="B45" s="0">
-        <v>0.66000000000000003</v>
-      </c>
-      <c r="C45" s="0" t="s">
+      <c r="B45">
+        <v>0.66</v>
+      </c>
+      <c r="C45" t="s">
         <v>44</v>
       </c>
-      <c r="D45" s="0" t="s">
+      <c r="D45" t="s">
         <v>64</v>
       </c>
-      <c r="E45" s="0" t="s">
+      <c r="E45" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="0" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A46" t="s">
         <v>105</v>
       </c>
-      <c r="B46" s="0">
+      <c r="B46">
         <v>5</v>
       </c>
-      <c r="C46" s="0" t="s">
+      <c r="C46" t="s">
         <v>111</v>
       </c>
-      <c r="D46" s="0" t="s">
+      <c r="D46" t="s">
         <v>113</v>
       </c>
-      <c r="E46" s="0" t="s">
+      <c r="E46" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="0" t="s">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A47" t="s">
         <v>106</v>
       </c>
-      <c r="B47" s="0">
+      <c r="B47">
         <v>50</v>
       </c>
-      <c r="C47" s="0" t="s">
+      <c r="C47" t="s">
         <v>112</v>
       </c>
-      <c r="D47" s="0" t="s">
+      <c r="D47" t="s">
         <v>64</v>
       </c>
-      <c r="E47" s="0" t="s">
+      <c r="E47" t="s">
         <v>121</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Claude 2nd pass for new input data format
</commit_message>
<xml_diff>
--- a/VehicleParameters.xlsx
+++ b/VehicleParameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\GitHub\RIT_RacingBrakesAnalysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B495F0F-15FE-490D-AC2A-5AE6B27A8A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8406F1E-332E-45A1-ACD6-C7E8ABCAA152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-86" yWindow="0" windowWidth="11143" windowHeight="13080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameters" sheetId="1" r:id="rId1"/>
@@ -34,86 +34,224 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="208">
   <si>
     <t>Name</t>
   </si>
   <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Units</t>
+  </si>
+  <si>
+    <t>Basis</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
     <t>VehicleMass</t>
   </si>
   <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>whole vehicle</t>
+  </si>
+  <si>
+    <t>As-driven mass.</t>
+  </si>
+  <si>
     <t>I_corner</t>
   </si>
   <si>
+    <t>kg*m^2</t>
+  </si>
+  <si>
+    <t>single corner</t>
+  </si>
+  <si>
+    <t>Rotational inertia of ONE corner (wheel+tire+hub+rotor). Equivalent rotating mass = I/WheelR^2</t>
+  </si>
+  <si>
     <t>WheelR</t>
   </si>
   <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>Loaded rolling radius.</t>
+  </si>
+  <si>
     <t>gear_ratio</t>
   </si>
   <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Motor to wheel gear ratio.</t>
+  </si>
+  <si>
     <t>TambC_fallback</t>
   </si>
   <si>
+    <t>degC</t>
+  </si>
+  <si>
+    <t>ambient</t>
+  </si>
+  <si>
+    <t>Fallback only; each dataset derives its own ambient from first rotor temps.</t>
+  </si>
+  <si>
     <t>RotorMass_front</t>
   </si>
   <si>
+    <t>single rotor</t>
+  </si>
+  <si>
+    <t>Mass of ONE front rotor.</t>
+  </si>
+  <si>
     <t>RotorMass_rear</t>
   </si>
   <si>
+    <t>Mass of ONE rear rotor.</t>
+  </si>
+  <si>
     <t>RotorArea_front</t>
   </si>
   <si>
+    <t>m^2</t>
+  </si>
+  <si>
+    <t>Convective surface area of ONE front rotor.</t>
+  </si>
+  <si>
     <t>RotorArea_rear</t>
   </si>
   <si>
+    <t>Convective surface area of ONE rear rotor.</t>
+  </si>
+  <si>
     <t>front_rotor_dia</t>
   </si>
   <si>
+    <t>Reference geometry only. NOT used as the friction lever arm (see front_pad_mean_radius).</t>
+  </si>
+  <si>
     <t>rear_rotor_dia</t>
   </si>
   <si>
     <t>A_pad_front</t>
   </si>
   <si>
+    <t>mm^2</t>
+  </si>
+  <si>
+    <t>single pad</t>
+  </si>
+  <si>
+    <t>Contact area of ONE front pad. x2 = one corner, x4 = one axle.</t>
+  </si>
+  <si>
     <t>A_pad_rear</t>
   </si>
   <si>
+    <t>Contact area of ONE rear pad.</t>
+  </si>
+  <si>
     <t>pads_per_corner</t>
   </si>
   <si>
+    <t>count</t>
+  </si>
+  <si>
+    <t>Pads rubbing one rotor (both sides of the disc).</t>
+  </si>
+  <si>
     <t>front_pad_mean_radius</t>
   </si>
   <si>
+    <t>Friction lever arm of front pad</t>
+  </si>
+  <si>
     <t>rear_pad_mean_radius</t>
   </si>
   <si>
+    <t>Friction lever arm of rear pad</t>
+  </si>
+  <si>
     <t>front_piston_count</t>
   </si>
   <si>
+    <t>single caliper (total)</t>
+  </si>
+  <si>
+    <t>ALL pistons in one front caliper, both sides combined.</t>
+  </si>
+  <si>
     <t>rear_piston_count</t>
   </si>
   <si>
+    <t>ALL pistons in one rear caliper, both sides combined.</t>
+  </si>
+  <si>
     <t>front_piston_dia</t>
   </si>
   <si>
+    <t>single piston</t>
+  </si>
+  <si>
+    <t>Bore diameter of ONE front piston.</t>
+  </si>
+  <si>
     <t>rear_piston_dia</t>
   </si>
   <si>
+    <t>Bore diameter of ONE rear piston.</t>
+  </si>
+  <si>
     <t>front_caliper_opposed</t>
   </si>
   <si>
+    <t>bool</t>
+  </si>
+  <si>
+    <t>single caliper</t>
+  </si>
+  <si>
+    <t>1 = opposed/fixed (pistons split evenly both sides, clamp force uses half the count). 0 = floating (all pistons one side).</t>
+  </si>
+  <si>
     <t>rear_caliper_opposed</t>
   </si>
   <si>
+    <t>As above.</t>
+  </si>
+  <si>
     <t>BrakeFrac</t>
   </si>
   <si>
+    <t>model calibration</t>
+  </si>
+  <si>
+    <t>Mechanical brake fraction (total energy - drivetrain/other losses)</t>
+  </si>
+  <si>
     <t>CalibrationFactor</t>
   </si>
   <si>
+    <t>Empirical thermal derating, "fudge factor"</t>
+  </si>
+  <si>
     <t>aero_open_a</t>
   </si>
   <si>
+    <t>DRS open: F = a*mph^2 + b*mph + c.</t>
+  </si>
+  <si>
     <t>aero_open_b</t>
   </si>
   <si>
@@ -123,6 +261,9 @@
     <t>aero_closed_a</t>
   </si>
   <si>
+    <t>DRS closed.</t>
+  </si>
+  <si>
     <t>aero_closed_b</t>
   </si>
   <si>
@@ -132,274 +273,391 @@
     <t>press_front_slope</t>
   </si>
   <si>
+    <t>psi/ADC</t>
+  </si>
+  <si>
+    <t>sensor</t>
+  </si>
+  <si>
+    <t>frontpressure = max(slope*adc - offset, 0).</t>
+  </si>
+  <si>
     <t>press_front_offset</t>
   </si>
   <si>
+    <t>psi</t>
+  </si>
+  <si>
     <t>press_rear_slope</t>
   </si>
   <si>
+    <t>rearpressure = max(slope*adc - offset, 0).</t>
+  </si>
+  <si>
     <t>press_rear_offset</t>
   </si>
   <si>
     <t>temp_adc_slope</t>
   </si>
   <si>
+    <t>degC/ADC</t>
+  </si>
+  <si>
+    <t>temp_C = slope*(adc - offset).</t>
+  </si>
+  <si>
     <t>temp_adc_offset</t>
   </si>
   <si>
+    <t>ADC</t>
+  </si>
+  <si>
     <t>velx_threshold</t>
   </si>
   <si>
+    <t>m/s</t>
+  </si>
+  <si>
+    <t>Velocity cleaning threshold; readings above this are zeroed.</t>
+  </si>
+  <si>
     <t>min_pressure</t>
   </si>
   <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Units</t>
-  </si>
-  <si>
-    <t>kg</t>
-  </si>
-  <si>
-    <t>kg*m^2</t>
-  </si>
-  <si>
-    <t>m</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>degC</t>
-  </si>
-  <si>
-    <t>m^2</t>
-  </si>
-  <si>
-    <t>mm^2</t>
-  </si>
-  <si>
-    <t>count</t>
-  </si>
-  <si>
-    <t>bool</t>
-  </si>
-  <si>
-    <t>psi/ADC</t>
-  </si>
-  <si>
-    <t>psi</t>
-  </si>
-  <si>
-    <t>degC/ADC</t>
-  </si>
-  <si>
-    <t>ADC</t>
-  </si>
-  <si>
-    <t>m/s</t>
-  </si>
-  <si>
-    <t>Basis</t>
-  </si>
-  <si>
-    <t>whole vehicle</t>
-  </si>
-  <si>
-    <t>single corner</t>
-  </si>
-  <si>
-    <t>ambient</t>
-  </si>
-  <si>
-    <t>single rotor</t>
-  </si>
-  <si>
-    <t>single pad</t>
-  </si>
-  <si>
-    <t>single caliper (total)</t>
-  </si>
-  <si>
-    <t>single piston</t>
-  </si>
-  <si>
-    <t>single caliper</t>
-  </si>
-  <si>
-    <t>model calibration</t>
-  </si>
-  <si>
-    <t>sensor</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Loaded rolling radius.</t>
-  </si>
-  <si>
-    <t>Motor to wheel gear ratio.</t>
-  </si>
-  <si>
-    <t>Fallback only; each dataset derives its own ambient from first rotor temps.</t>
-  </si>
-  <si>
-    <t>Mass of ONE front rotor.</t>
-  </si>
-  <si>
-    <t>Mass of ONE rear rotor.</t>
-  </si>
-  <si>
-    <t>Convective surface area of ONE front rotor.</t>
-  </si>
-  <si>
-    <t>Reference geometry only. NOT used as the friction lever arm (see front_pad_mean_radius).</t>
-  </si>
-  <si>
-    <t>Contact area of ONE front pad. x2 = one corner, x4 = one axle.</t>
-  </si>
-  <si>
-    <t>Contact area of ONE rear pad.</t>
-  </si>
-  <si>
-    <t>Pads rubbing one rotor (both sides of the disc).</t>
-  </si>
-  <si>
-    <t>ALL pistons in one front caliper, both sides combined.</t>
-  </si>
-  <si>
-    <t>ALL pistons in one rear caliper, both sides combined.</t>
-  </si>
-  <si>
-    <t>Bore diameter of ONE front piston.</t>
-  </si>
-  <si>
-    <t>Bore diameter of ONE rear piston.</t>
-  </si>
-  <si>
-    <t>1 = opposed/fixed (pistons split evenly both sides, clamp force uses half the count). 0 = floating (all pistons one side).</t>
-  </si>
-  <si>
-    <t>As above.</t>
-  </si>
-  <si>
-    <t>DRS open: F = a*mph^2 + b*mph + c.</t>
-  </si>
-  <si>
-    <t>DRS closed.</t>
-  </si>
-  <si>
-    <t>frontpressure = max(slope*adc - offset, 0).</t>
-  </si>
-  <si>
-    <t>rearpressure = max(slope*adc - offset, 0).</t>
-  </si>
-  <si>
-    <t>temp_C = slope*(adc - offset).</t>
-  </si>
-  <si>
-    <t>Velocity cleaning threshold; readings above this are zeroed.</t>
-  </si>
-  <si>
     <t>Threshold to consider a corner's brake engaged.</t>
   </si>
   <si>
+    <t>current_limit_actual</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>vehicle setting</t>
+  </si>
+  <si>
+    <t>Motor controller current limit the loaded data was recorded at. Predicted-regen curves scale by current_limit/current_limit_actual.</t>
+  </si>
+  <si>
+    <t>torque_limit_total_MN</t>
+  </si>
+  <si>
+    <t>%Mn</t>
+  </si>
+  <si>
+    <t>Maximum observed total motor torque command, all 4 wheels combined. Wheel-side limit = value/100*9.8*gear_ratio.</t>
+  </si>
+  <si>
+    <t>regen_power_limit</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>Motor controller regen power limit.</t>
+  </si>
+  <si>
+    <t>regen_max_curve_a</t>
+  </si>
+  <si>
+    <t>Nm</t>
+  </si>
+  <si>
+    <t>Max regen wheel torque curve: T = a*mph^b, before efficiency and current-limit scaling.</t>
+  </si>
+  <si>
+    <t>regen_max_curve_b</t>
+  </si>
+  <si>
+    <t>Exponent of the max regen wheel torque curve (negative: available torque falls with speed).</t>
+  </si>
+  <si>
+    <t>regen_efficiency</t>
+  </si>
+  <si>
+    <t>Utilization factor applied to the theoretical max regen curve to match measured data.</t>
+  </si>
+  <si>
+    <t>min_regen_speed</t>
+  </si>
+  <si>
+    <t>mph</t>
+  </si>
+  <si>
+    <t>Minimum vehicle speed for regen; below this the system recovers no energy.</t>
+  </si>
+  <si>
+    <t>min_energy_threshold</t>
+  </si>
+  <si>
+    <t>kJ</t>
+  </si>
+  <si>
+    <t>Minimum cumulative regen energy before the predicted-vs-actual percent difference is reported (avoids a near-zero denominator early in a run).</t>
+  </si>
+  <si>
+    <t>rho_rotor</t>
+  </si>
+  <si>
+    <t>kg/m^3</t>
+  </si>
+  <si>
+    <t>rotor design</t>
+  </si>
+  <si>
+    <t>Rotor density (4130 steel value used in BrakeCoeffOptimizer.m).</t>
+  </si>
+  <si>
+    <t>hw_x1_front</t>
+  </si>
+  <si>
+    <t>W/m^2K per m/s</t>
+  </si>
+  <si>
+    <t>h_w = x1*v + b1, front. Seed value from BrakeCoeffOptimizer.m. REPLACE with your final fit.</t>
+  </si>
+  <si>
+    <t>hw_b1_front</t>
+  </si>
+  <si>
+    <t>W/m^2K</t>
+  </si>
+  <si>
+    <t>Seed value. REPLACE with your final fit.</t>
+  </si>
+  <si>
+    <t>hw_x1_rear</t>
+  </si>
+  <si>
+    <t>hw_b1_rear</t>
+  </si>
+  <si>
+    <t>padfrac_x2</t>
+  </si>
+  <si>
+    <t>1/K</t>
+  </si>
+  <si>
+    <t>PadFrac(T_K) = x2*T_K + b2, clamped to [0,1]. Seed value. REPLACE with your final fit.</t>
+  </si>
+  <si>
+    <t>padfrac_b2</t>
+  </si>
+  <si>
+    <t>Tbias_front</t>
+  </si>
+  <si>
+    <t>regen_front_frac_a</t>
+  </si>
+  <si>
+    <t>rotor design (legacy)</t>
+  </si>
+  <si>
+    <t>Front share of vehicle regen power vs speed, ff = a + b*v_mps. Only used by the LEGACY torque-based drive-cycle format; the force-based format measures friction heat directly and does not need this.</t>
+  </si>
+  <si>
+    <t>regen_front_frac_b</t>
+  </si>
+  <si>
+    <t>1/(m/s)</t>
+  </si>
+  <si>
+    <t>Speed slope of the regen front share. Legacy format only (see regen_front_frac_a).</t>
+  </si>
+  <si>
+    <t>min_pedal_force_N</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Threshold on the legacy friction_brake_force_N pedal-force column. Not used by the force-based format (which gates on RequiredBrakingMagnitude_N &gt; 0).</t>
+  </si>
+  <si>
+    <t>T_target_F</t>
+  </si>
+  <si>
+    <t>degF</t>
+  </si>
+  <si>
+    <t>T_init_F</t>
+  </si>
+  <si>
+    <t>Initial rotor temperature. Set to ambient (TambC_fallback = 77.0 degF) unless stated otherwise.</t>
+  </si>
+  <si>
+    <t>Do_front_mm</t>
+  </si>
+  <si>
+    <t>mm</t>
+  </si>
+  <si>
+    <t>Fixed outer diameter, front.</t>
+  </si>
+  <si>
+    <t>Di_front_mm</t>
+  </si>
+  <si>
+    <t>Fixed inner diameter, front. Radial width = 19.05 mm.</t>
+  </si>
+  <si>
+    <t>t_min_front_mm</t>
+  </si>
+  <si>
+    <t>Thickness lower limit, front.</t>
+  </si>
+  <si>
+    <t>t_max_front_mm</t>
+  </si>
+  <si>
+    <t>Thickness upper limit, front.</t>
+  </si>
+  <si>
+    <t>s_min_front_mm</t>
+  </si>
+  <si>
+    <t>Min feature size (hole dia. / slot width), front.</t>
+  </si>
+  <si>
+    <t>phi_max_front</t>
+  </si>
+  <si>
+    <t>Max removed face-area fraction, front (may be reduced further by pattern packing - see enforce_pattern_packing).</t>
+  </si>
+  <si>
+    <t>cut_type_front</t>
+  </si>
+  <si>
+    <t>1=hole/2=slot</t>
+  </si>
+  <si>
+    <t>1 = drilled circular holes (L_max = 4*Ar/s_min); 2 = long slots (L_max = 2*Ar/s_min).</t>
+  </si>
+  <si>
+    <t>Do_rear_mm</t>
+  </si>
+  <si>
+    <t>Fixed outer diameter, rear.</t>
+  </si>
+  <si>
+    <t>Di_rear_mm</t>
+  </si>
+  <si>
+    <t>Fixed inner diameter, rear. Radial width = 22.86 mm.</t>
+  </si>
+  <si>
+    <t>t_min_rear_mm</t>
+  </si>
+  <si>
+    <t>Thickness lower limit, rear.</t>
+  </si>
+  <si>
+    <t>t_max_rear_mm</t>
+  </si>
+  <si>
+    <t>Thickness upper limit, rear.</t>
+  </si>
+  <si>
+    <t>s_min_rear_mm</t>
+  </si>
+  <si>
+    <t>Min feature size, rear.</t>
+  </si>
+  <si>
+    <t>phi_max_rear</t>
+  </si>
+  <si>
+    <t>Max removed face-area fraction, rear.</t>
+  </si>
+  <si>
+    <t>cut_type_rear</t>
+  </si>
+  <si>
+    <t>1 = drilled circular holes; 2 = long slots.</t>
+  </si>
+  <si>
+    <t>include_edge_area</t>
+  </si>
+  <si>
+    <t>0/1</t>
+  </si>
+  <si>
+    <t>1 = RotorArea includes the inner/outer cylindrical edges, pi*(Do+Di)*t. 0 = faces + cut walls only.</t>
+  </si>
+  <si>
+    <t>edge_margin_mm</t>
+  </si>
+  <si>
+    <t>Radial material margin a cut pattern must leave at BOTH the OD and the ID.</t>
+  </si>
+  <si>
+    <t>enforce_pattern_packing</t>
+  </si>
+  <si>
+    <t>1 = cap phi_max at what a real single-row cut pattern can deliver (the front rotor is packing-limited to ~0.483 vs the 0.500 spec at this radial width). 0 = use phi_max as specified.</t>
+  </si>
+  <si>
+    <t>drs_state</t>
+  </si>
+  <si>
+    <t>CONFIRM. 0 = closed, 1 = open. Only used by the LEGACY format, which has no AeroDragMagnitude_N column and must compute aero force from the aero_* polynomial instead.</t>
+  </si>
+  <si>
+    <t>use_dt_s_column</t>
+  </si>
+  <si>
+    <t>1 = build the time base from dt_s (needed because the legacy time column saturates at 3 sig figs above 1000 s). Only used by the LEGACY format; the force-based format uses Time_s directly.</t>
+  </si>
+  <si>
+    <t>exclude_lap_artifacts</t>
+  </si>
+  <si>
+    <t>1 = force the passive-cooling branch on the two artifact rows at each legacy-format lap start. The force-based format uses the explicit Lap column instead and has no artifact rows.</t>
+  </si>
+  <si>
+    <t>n_mass_grid</t>
+  </si>
+  <si>
+    <t>solver setting</t>
+  </si>
+  <si>
+    <t>Number of masses spanning the achievable envelope for the frontier and trade-off table.</t>
+  </si>
+  <si>
+    <t>A_bracket_lo</t>
+  </si>
+  <si>
+    <t>Lower bracket for the area root-find.</t>
+  </si>
+  <si>
+    <t>A_bracket_hi</t>
+  </si>
+  <si>
+    <t>Upper bracket for the area root-find.</t>
+  </si>
+  <si>
+    <t>area_bisect_iters</t>
+  </si>
+  <si>
+    <t>Bisection iterations on area (40 reaches machine precision on this bracket).</t>
+  </si>
+  <si>
+    <t>euler_warn_threshold</t>
+  </si>
+  <si>
+    <t>Warn if max(dt*h_w*A/(m*cp)) exceeds this (explicit-Euler stability margin).</t>
+  </si>
+  <si>
     <t>Temp_F</t>
   </si>
   <si>
     <t>Mu</t>
   </si>
   <si>
-    <t>Rotational inertia of ONE corner (wheel+tire+hub+rotor). Equivalent rotating mass = I/WheelR^2</t>
-  </si>
-  <si>
-    <t>As-driven mass.</t>
-  </si>
-  <si>
-    <t>Convective surface area of ONE rear rotor.</t>
-  </si>
-  <si>
-    <t>Friction lever arm of front pad</t>
-  </si>
-  <si>
-    <t>Friction lever arm of rear pad</t>
-  </si>
-  <si>
-    <t>Mechanical brake fraction (total energy - drivetrain/other losses)</t>
-  </si>
-  <si>
-    <t>Empirical thermal derating, "fudge factor"</t>
-  </si>
-  <si>
-    <t>current_limit_actual</t>
-  </si>
-  <si>
-    <t>torque_limit_total_MN</t>
-  </si>
-  <si>
-    <t>regen_power_limit</t>
-  </si>
-  <si>
-    <t>regen_max_curve_a</t>
-  </si>
-  <si>
-    <t>regen_max_curve_b</t>
-  </si>
-  <si>
-    <t>regen_efficiency</t>
-  </si>
-  <si>
-    <t>min_regen_speed</t>
-  </si>
-  <si>
-    <t>min_energy_threshold</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>%Mn</t>
-  </si>
-  <si>
-    <t>W</t>
-  </si>
-  <si>
-    <t>Nm</t>
-  </si>
-  <si>
-    <t>mph</t>
-  </si>
-  <si>
-    <t>kJ</t>
-  </si>
-  <si>
-    <t>vehicle setting</t>
-  </si>
-  <si>
-    <t>Motor controller current limit the loaded data was recorded at. Predicted-regen curves scale by current_limit/current_limit_actual.</t>
-  </si>
-  <si>
-    <t>Maximum observed total motor torque command, all 4 wheels combined. Wheel-side limit = value/100*9.8*gear_ratio.</t>
-  </si>
-  <si>
-    <t>Motor controller regen power limit.</t>
-  </si>
-  <si>
-    <t>Max regen wheel torque curve: T = a*mph^b, before efficiency and current-limit scaling.</t>
-  </si>
-  <si>
-    <t>Exponent of the max regen wheel torque curve (negative: available torque falls with speed).</t>
-  </si>
-  <si>
-    <t>Utilization factor applied to the theoretical max regen curve to match measured data.</t>
-  </si>
-  <si>
-    <t>Minimum vehicle speed for regen; below this the system recovers no energy.</t>
-  </si>
-  <si>
-    <t>Minimum cumulative regen energy before the predicted-vs-actual percent difference is reported (avoids a near-zero denominator early in a run).</t>
+    <t>Front fraction of FRICTION braking force (FrictionBrakeForce_N); rear uses 1-Tbias_front.</t>
+  </si>
+  <si>
+    <t>Peak rotor temperature not to be exceeded over the whole run.</t>
   </si>
 </sst>
 </file>
@@ -437,9 +695,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -774,7 +1042,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="21.3046875" customWidth="1"/>
@@ -789,774 +1057,1420 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>55</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>66</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B2">
         <v>259</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>93</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B3">
         <v>0.11</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>92</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="B4">
         <v>0.21299999999999999</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>67</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B5">
         <v>12.97</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="B6">
         <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>69</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="B7">
         <v>0.51070000000000004</v>
       </c>
       <c r="C7" t="s">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="E7" t="s">
-        <v>70</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="B8">
         <v>0.33429999999999999</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>71</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B9">
         <v>3.7999999999999999E-2</v>
       </c>
       <c r="C9" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="D9" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="B10">
         <v>2.2599999999999999E-2</v>
       </c>
       <c r="C10" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="D10" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>94</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="B11">
         <v>0.20574000000000001</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="D11" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="E11" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="B12">
         <v>0.20574000000000001</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="D12" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="B13">
         <v>1520</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="D13" t="s">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="E13" t="s">
-        <v>74</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="B14">
         <v>650</v>
       </c>
       <c r="C14" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="D14" t="s">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="E14" t="s">
-        <v>75</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="B15">
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>76</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="B16">
         <v>9.2710000000000001E-2</v>
       </c>
       <c r="C16" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="D16" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>95</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="B17">
         <v>9.3979999999999994E-2</v>
       </c>
       <c r="C17" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="D17" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>96</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="B18">
         <v>6</v>
       </c>
       <c r="C18" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D18" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="E18" t="s">
-        <v>77</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="B19">
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D19" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="E19" t="s">
-        <v>78</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>54</v>
       </c>
       <c r="B20">
         <v>1.57226E-2</v>
       </c>
       <c r="C20" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="D20" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="E20" t="s">
-        <v>79</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="B21">
         <v>1.41732E-2</v>
       </c>
       <c r="C21" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="D21" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="E21" t="s">
-        <v>80</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
-        <v>21</v>
+        <v>59</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D22" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E22" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="D23" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E23" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="B24">
         <v>0.82</v>
       </c>
       <c r="C24" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="D24" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>97</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>68</v>
       </c>
       <c r="B25">
         <v>0.8</v>
       </c>
       <c r="C25" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="D25" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="B26">
         <v>7.9302399999999995E-2</v>
       </c>
       <c r="C26" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="D26" t="s">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="E26" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="B27">
         <v>1.4648300000000001</v>
       </c>
       <c r="C27" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="D27" t="s">
-        <v>56</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="B28">
         <v>-37.239930000000001</v>
       </c>
       <c r="C28" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="D28" t="s">
-        <v>56</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="B29">
         <v>0.13624700000000001</v>
       </c>
       <c r="C29" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="D29" t="s">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="E29" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="B30">
         <v>2.5344899999999999</v>
       </c>
       <c r="C30" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="D30" t="s">
-        <v>56</v>
+        <v>7</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="B31">
         <v>-67.449749999999995</v>
       </c>
       <c r="C31" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="D31" t="s">
-        <v>56</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
-        <v>31</v>
+        <v>78</v>
       </c>
       <c r="B32">
         <v>0.92400000000000004</v>
       </c>
       <c r="C32" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="D32" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="E32" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
-        <v>32</v>
+        <v>82</v>
       </c>
       <c r="B33">
         <v>332.64</v>
       </c>
       <c r="C33" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="D33" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="B34">
         <v>0.92400000000000004</v>
       </c>
       <c r="C34" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="D34" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="E34" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
-        <v>34</v>
+        <v>86</v>
       </c>
       <c r="B35">
         <v>376.06799999999998</v>
       </c>
       <c r="C35" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="D35" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
-        <v>35</v>
+        <v>87</v>
       </c>
       <c r="B36">
         <v>0.246</v>
       </c>
       <c r="C36" t="s">
-        <v>52</v>
+        <v>88</v>
       </c>
       <c r="D36" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="E36" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
-        <v>36</v>
+        <v>90</v>
       </c>
       <c r="B37">
         <v>406</v>
       </c>
       <c r="C37" t="s">
-        <v>53</v>
+        <v>91</v>
       </c>
       <c r="D37" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
-        <v>37</v>
+        <v>92</v>
       </c>
       <c r="B38">
         <v>34</v>
       </c>
       <c r="C38" t="s">
-        <v>54</v>
+        <v>93</v>
       </c>
       <c r="D38" t="s">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="E38" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
-        <v>38</v>
+        <v>95</v>
       </c>
       <c r="B39">
         <v>5</v>
       </c>
       <c r="C39" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="D39" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E39" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B40">
         <v>35</v>
       </c>
       <c r="C40" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="D40" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="E40" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B41">
         <v>200</v>
       </c>
       <c r="C41" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="D41" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="E41" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B42">
         <v>30000</v>
       </c>
       <c r="C42" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D42" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="E42" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B43">
         <v>7041</v>
       </c>
       <c r="C43" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D43" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E43" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B44">
         <v>-0.93500000000000005</v>
       </c>
       <c r="C44" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="D44" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E44" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="B45">
         <v>0.66</v>
       </c>
       <c r="C45" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="D45" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E45" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="B46">
         <v>5</v>
       </c>
       <c r="C46" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D46" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="E46" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="B47">
         <v>50</v>
       </c>
       <c r="C47" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="D47" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E47" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A48" t="s">
+        <v>120</v>
+      </c>
+      <c r="B48">
+        <v>7850</v>
+      </c>
+      <c r="C48" t="s">
         <v>121</v>
+      </c>
+      <c r="D48" t="s">
+        <v>122</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A49" t="s">
+        <v>124</v>
+      </c>
+      <c r="B49">
+        <v>2.3669020000000001</v>
+      </c>
+      <c r="C49" t="s">
+        <v>125</v>
+      </c>
+      <c r="D49" t="s">
+        <v>66</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A50" t="s">
+        <v>127</v>
+      </c>
+      <c r="B50">
+        <v>21.133071999999999</v>
+      </c>
+      <c r="C50" t="s">
+        <v>128</v>
+      </c>
+      <c r="D50" t="s">
+        <v>66</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A51" t="s">
+        <v>130</v>
+      </c>
+      <c r="B51">
+        <v>3.6413859999999998</v>
+      </c>
+      <c r="C51" t="s">
+        <v>125</v>
+      </c>
+      <c r="D51" t="s">
+        <v>66</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A52" t="s">
+        <v>131</v>
+      </c>
+      <c r="B52">
+        <v>29.359404999999999</v>
+      </c>
+      <c r="C52" t="s">
+        <v>128</v>
+      </c>
+      <c r="D52" t="s">
+        <v>66</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A53" t="s">
+        <v>132</v>
+      </c>
+      <c r="B53">
+        <v>4.6090397E-4</v>
+      </c>
+      <c r="C53" t="s">
+        <v>133</v>
+      </c>
+      <c r="D53" t="s">
+        <v>66</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A54" t="s">
+        <v>135</v>
+      </c>
+      <c r="B54">
+        <v>0.13389237000000001</v>
+      </c>
+      <c r="C54" t="s">
+        <v>17</v>
+      </c>
+      <c r="D54" t="s">
+        <v>66</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A55" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B55" s="3">
+        <v>0.65</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A56" t="s">
+        <v>137</v>
+      </c>
+      <c r="B56">
+        <v>0.5</v>
+      </c>
+      <c r="C56" t="s">
+        <v>17</v>
+      </c>
+      <c r="D56" t="s">
+        <v>138</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A57" t="s">
+        <v>140</v>
+      </c>
+      <c r="B57">
+        <v>6.6666666666666671E-3</v>
+      </c>
+      <c r="C57" t="s">
+        <v>141</v>
+      </c>
+      <c r="D57" t="s">
+        <v>138</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A58" t="s">
+        <v>143</v>
+      </c>
+      <c r="B58">
+        <v>0</v>
+      </c>
+      <c r="C58" t="s">
+        <v>144</v>
+      </c>
+      <c r="D58" t="s">
+        <v>138</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A59" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="B59" s="3">
+        <v>800</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A60" t="s">
+        <v>148</v>
+      </c>
+      <c r="B60">
+        <v>77</v>
+      </c>
+      <c r="C60" t="s">
+        <v>147</v>
+      </c>
+      <c r="D60" t="s">
+        <v>122</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A61" t="s">
+        <v>150</v>
+      </c>
+      <c r="B61">
+        <v>204.47</v>
+      </c>
+      <c r="C61" t="s">
+        <v>151</v>
+      </c>
+      <c r="D61" t="s">
+        <v>122</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A62" t="s">
+        <v>153</v>
+      </c>
+      <c r="B62">
+        <v>166.37</v>
+      </c>
+      <c r="C62" t="s">
+        <v>151</v>
+      </c>
+      <c r="D62" t="s">
+        <v>122</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A63" t="s">
+        <v>155</v>
+      </c>
+      <c r="B63">
+        <v>2.54</v>
+      </c>
+      <c r="C63" t="s">
+        <v>151</v>
+      </c>
+      <c r="D63" t="s">
+        <v>122</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A64" t="s">
+        <v>157</v>
+      </c>
+      <c r="B64">
+        <v>5.08</v>
+      </c>
+      <c r="C64" t="s">
+        <v>151</v>
+      </c>
+      <c r="D64" t="s">
+        <v>122</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A65" t="s">
+        <v>159</v>
+      </c>
+      <c r="B65">
+        <v>2.54</v>
+      </c>
+      <c r="C65" t="s">
+        <v>151</v>
+      </c>
+      <c r="D65" t="s">
+        <v>122</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A66" t="s">
+        <v>161</v>
+      </c>
+      <c r="B66">
+        <v>0.5</v>
+      </c>
+      <c r="C66" t="s">
+        <v>17</v>
+      </c>
+      <c r="D66" t="s">
+        <v>122</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A67" t="s">
+        <v>163</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>164</v>
+      </c>
+      <c r="D67" t="s">
+        <v>122</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A68" t="s">
+        <v>166</v>
+      </c>
+      <c r="B68">
+        <v>195.58</v>
+      </c>
+      <c r="C68" t="s">
+        <v>151</v>
+      </c>
+      <c r="D68" t="s">
+        <v>122</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A69" t="s">
+        <v>168</v>
+      </c>
+      <c r="B69">
+        <v>149.86000000000001</v>
+      </c>
+      <c r="C69" t="s">
+        <v>151</v>
+      </c>
+      <c r="D69" t="s">
+        <v>122</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A70" t="s">
+        <v>170</v>
+      </c>
+      <c r="B70">
+        <v>2.54</v>
+      </c>
+      <c r="C70" t="s">
+        <v>151</v>
+      </c>
+      <c r="D70" t="s">
+        <v>122</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A71" t="s">
+        <v>172</v>
+      </c>
+      <c r="B71">
+        <v>5.08</v>
+      </c>
+      <c r="C71" t="s">
+        <v>151</v>
+      </c>
+      <c r="D71" t="s">
+        <v>122</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A72" t="s">
+        <v>174</v>
+      </c>
+      <c r="B72">
+        <v>2.54</v>
+      </c>
+      <c r="C72" t="s">
+        <v>151</v>
+      </c>
+      <c r="D72" t="s">
+        <v>122</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A73" t="s">
+        <v>176</v>
+      </c>
+      <c r="B73">
+        <v>0.5</v>
+      </c>
+      <c r="C73" t="s">
+        <v>17</v>
+      </c>
+      <c r="D73" t="s">
+        <v>122</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A74" t="s">
+        <v>178</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>164</v>
+      </c>
+      <c r="D74" t="s">
+        <v>122</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A75" t="s">
+        <v>180</v>
+      </c>
+      <c r="B75">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>181</v>
+      </c>
+      <c r="D75" t="s">
+        <v>122</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A76" t="s">
+        <v>183</v>
+      </c>
+      <c r="B76">
+        <v>2.54</v>
+      </c>
+      <c r="C76" t="s">
+        <v>151</v>
+      </c>
+      <c r="D76" t="s">
+        <v>122</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A77" t="s">
+        <v>185</v>
+      </c>
+      <c r="B77">
+        <v>1</v>
+      </c>
+      <c r="C77" t="s">
+        <v>181</v>
+      </c>
+      <c r="D77" t="s">
+        <v>122</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A78" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B78" s="3">
+        <v>0</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E78" s="5" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A79" t="s">
+        <v>189</v>
+      </c>
+      <c r="B79">
+        <v>1</v>
+      </c>
+      <c r="C79" t="s">
+        <v>181</v>
+      </c>
+      <c r="D79" t="s">
+        <v>138</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A80" t="s">
+        <v>191</v>
+      </c>
+      <c r="B80">
+        <v>1</v>
+      </c>
+      <c r="C80" t="s">
+        <v>181</v>
+      </c>
+      <c r="D80" t="s">
+        <v>138</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A81" t="s">
+        <v>193</v>
+      </c>
+      <c r="B81">
+        <v>61</v>
+      </c>
+      <c r="C81" t="s">
+        <v>43</v>
+      </c>
+      <c r="D81" t="s">
+        <v>194</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A82" t="s">
+        <v>196</v>
+      </c>
+      <c r="B82">
+        <v>1E-4</v>
+      </c>
+      <c r="C82" t="s">
+        <v>29</v>
+      </c>
+      <c r="D82" t="s">
+        <v>194</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A83" t="s">
+        <v>198</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83" t="s">
+        <v>29</v>
+      </c>
+      <c r="D83" t="s">
+        <v>194</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A84" t="s">
+        <v>200</v>
+      </c>
+      <c r="B84">
+        <v>40</v>
+      </c>
+      <c r="C84" t="s">
+        <v>43</v>
+      </c>
+      <c r="D84" t="s">
+        <v>194</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A85" t="s">
+        <v>202</v>
+      </c>
+      <c r="B85">
+        <v>0.2</v>
+      </c>
+      <c r="C85" t="s">
+        <v>17</v>
+      </c>
+      <c r="D85" t="s">
+        <v>194</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -1575,10 +2489,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>90</v>
+        <v>204</v>
       </c>
       <c r="B1" t="s">
-        <v>91</v>
+        <v>205</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.4">

</xml_diff>